<commit_message>
Update dashboard analytics and exports
</commit_message>
<xml_diff>
--- a/DMR_Monthly_Report.xlsx
+++ b/DMR_Monthly_Report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dashboards Projects\Follow-Up Sheets Dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dashboards Projects\Follow-Up Sheets Dashboard\follow-up-sheets-dashboard V3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62400EB8-A646-4C27-88D8-6A03386A7F40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16AB9E9D-083C-4D9E-8E84-9A7E5A447FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1000,9 +1000,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1063,6 +1060,114 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1105,90 +1210,6 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
@@ -1201,62 +1222,41 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1677,899 +1677,899 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="72"/>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-      <c r="P1" s="72"/>
-      <c r="Q1" s="72"/>
+      <c r="A1" s="30"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
     </row>
     <row r="2" spans="1:17" ht="100.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="73"/>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75"/>
-      <c r="D2" s="76" t="s">
+      <c r="A2" s="31"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
-      <c r="G2" s="77"/>
-      <c r="H2" s="77"/>
-      <c r="I2" s="77"/>
-      <c r="J2" s="77"/>
-      <c r="K2" s="77"/>
-      <c r="L2" s="77"/>
-      <c r="M2" s="77"/>
-      <c r="N2" s="78"/>
-      <c r="O2" s="79"/>
-      <c r="P2" s="80"/>
-      <c r="Q2" s="81"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="36"/>
+      <c r="O2" s="37"/>
+      <c r="P2" s="38"/>
+      <c r="Q2" s="39"/>
     </row>
     <row r="3" spans="1:17" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="82"/>
-      <c r="B3" s="82"/>
-      <c r="C3" s="82"/>
-      <c r="D3" s="82"/>
-      <c r="E3" s="82"/>
-      <c r="F3" s="82"/>
-      <c r="G3" s="82"/>
-      <c r="H3" s="82"/>
-      <c r="I3" s="82"/>
-      <c r="J3" s="82"/>
-      <c r="K3" s="82"/>
-      <c r="L3" s="82"/>
-      <c r="M3" s="82"/>
-      <c r="N3" s="82"/>
-      <c r="O3" s="82"/>
-      <c r="P3" s="82"/>
-      <c r="Q3" s="82"/>
+      <c r="A3" s="40"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+      <c r="K3" s="40"/>
+      <c r="L3" s="40"/>
+      <c r="M3" s="40"/>
+      <c r="N3" s="40"/>
+      <c r="O3" s="40"/>
+      <c r="P3" s="40"/>
+      <c r="Q3" s="40"/>
     </row>
     <row r="4" spans="1:17" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="83" t="s">
+      <c r="A4" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="84"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="84"/>
-      <c r="E4" s="85"/>
-      <c r="F4" s="85"/>
-      <c r="G4" s="85"/>
-      <c r="H4" s="85"/>
-      <c r="I4" s="85"/>
-      <c r="J4" s="85"/>
-      <c r="K4" s="85"/>
-      <c r="L4" s="85"/>
-      <c r="M4" s="85"/>
-      <c r="N4" s="85"/>
-      <c r="O4" s="85"/>
-      <c r="P4" s="84"/>
-      <c r="Q4" s="86"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="25"/>
+      <c r="N4" s="25"/>
+      <c r="O4" s="25"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="26"/>
     </row>
     <row r="5" spans="1:17" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="35"/>
-      <c r="C5" s="70"/>
-      <c r="D5" s="87"/>
-      <c r="E5" s="71" t="s">
+      <c r="B5" s="70"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="71"/>
-      <c r="G5" s="71"/>
-      <c r="H5" s="70" t="s">
+      <c r="F5" s="77"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="I5" s="70"/>
-      <c r="J5" s="70"/>
-      <c r="K5" s="70"/>
-      <c r="L5" s="70"/>
-      <c r="M5" s="70"/>
-      <c r="N5" s="70"/>
-      <c r="O5" s="70"/>
-      <c r="P5" s="66" t="s">
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
+      <c r="M5" s="27"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="Q5" s="68"/>
+      <c r="Q5" s="75"/>
     </row>
     <row r="6" spans="1:17" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="36"/>
-      <c r="B6" s="37"/>
-      <c r="C6" s="70"/>
-      <c r="D6" s="88"/>
-      <c r="E6" s="71"/>
-      <c r="F6" s="71"/>
-      <c r="G6" s="71"/>
-      <c r="H6" s="70"/>
-      <c r="I6" s="70"/>
-      <c r="J6" s="70"/>
-      <c r="K6" s="70"/>
-      <c r="L6" s="70"/>
-      <c r="M6" s="70"/>
-      <c r="N6" s="70"/>
-      <c r="O6" s="70"/>
-      <c r="P6" s="67"/>
-      <c r="Q6" s="69"/>
+      <c r="A6" s="71"/>
+      <c r="B6" s="72"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="77"/>
+      <c r="F6" s="77"/>
+      <c r="G6" s="77"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="27"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="27"/>
+      <c r="M6" s="27"/>
+      <c r="N6" s="27"/>
+      <c r="O6" s="27"/>
+      <c r="P6" s="74"/>
+      <c r="Q6" s="76"/>
     </row>
     <row r="7" spans="1:17" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="30"/>
-      <c r="B7" s="30"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30"/>
-      <c r="K7" s="30"/>
-      <c r="L7" s="30"/>
-      <c r="M7" s="30"/>
-      <c r="N7" s="30"/>
-      <c r="O7" s="30"/>
-      <c r="P7" s="30"/>
-      <c r="Q7" s="30"/>
+      <c r="A7" s="65"/>
+      <c r="B7" s="65"/>
+      <c r="C7" s="65"/>
+      <c r="D7" s="65"/>
+      <c r="E7" s="65"/>
+      <c r="F7" s="65"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="65"/>
+      <c r="I7" s="65"/>
+      <c r="J7" s="65"/>
+      <c r="K7" s="65"/>
+      <c r="L7" s="65"/>
+      <c r="M7" s="65"/>
+      <c r="N7" s="65"/>
+      <c r="O7" s="65"/>
+      <c r="P7" s="65"/>
+      <c r="Q7" s="65"/>
     </row>
     <row r="8" spans="1:17" ht="56.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="66" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="32"/>
-      <c r="J8" s="32"/>
-      <c r="K8" s="32"/>
-      <c r="L8" s="32"/>
-      <c r="M8" s="32"/>
-      <c r="N8" s="32"/>
-      <c r="O8" s="32"/>
-      <c r="P8" s="32"/>
-      <c r="Q8" s="33"/>
+      <c r="B8" s="67"/>
+      <c r="C8" s="67"/>
+      <c r="D8" s="67"/>
+      <c r="E8" s="67"/>
+      <c r="F8" s="67"/>
+      <c r="G8" s="67"/>
+      <c r="H8" s="67"/>
+      <c r="I8" s="67"/>
+      <c r="J8" s="67"/>
+      <c r="K8" s="67"/>
+      <c r="L8" s="67"/>
+      <c r="M8" s="67"/>
+      <c r="N8" s="67"/>
+      <c r="O8" s="67"/>
+      <c r="P8" s="67"/>
+      <c r="Q8" s="68"/>
     </row>
     <row r="9" spans="1:17" ht="70.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
     </row>
     <row r="10" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11">
+      <c r="A10" s="10">
         <v>1</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-      <c r="P10" s="7"/>
-      <c r="Q10" s="7"/>
+      <c r="C10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="6"/>
     </row>
     <row r="11" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="11">
+      <c r="A11" s="10">
         <v>2</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="7"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="7"/>
-      <c r="N11" s="7"/>
-      <c r="O11" s="7"/>
-      <c r="P11" s="7"/>
-      <c r="Q11" s="7"/>
+      <c r="C11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="6"/>
     </row>
     <row r="12" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11">
+      <c r="A12" s="10">
         <v>3</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="7"/>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="7"/>
+      <c r="C12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="6"/>
     </row>
     <row r="13" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="11">
+      <c r="A13" s="10">
         <v>4</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="7"/>
+      <c r="C13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
     </row>
     <row r="14" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="11">
+      <c r="A14" s="10">
         <v>5</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="7"/>
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
-      <c r="P14" s="7"/>
-      <c r="Q14" s="7"/>
+      <c r="C14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6"/>
     </row>
     <row r="15" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="11">
+      <c r="A15" s="10">
         <v>6</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="7"/>
-      <c r="N15" s="7"/>
-      <c r="O15" s="7"/>
-      <c r="P15" s="7"/>
-      <c r="Q15" s="7"/>
+      <c r="C15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="6"/>
     </row>
     <row r="16" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="11">
+      <c r="A16" s="10">
         <v>7</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F16" s="4"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="7"/>
-      <c r="N16" s="7"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="7"/>
-      <c r="Q16" s="7"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="6"/>
+      <c r="M16" s="6"/>
+      <c r="N16" s="6"/>
+      <c r="O16" s="6"/>
+      <c r="P16" s="6"/>
+      <c r="Q16" s="6"/>
     </row>
     <row r="17" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="11">
+      <c r="A17" s="10">
         <v>8</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7"/>
-      <c r="M17" s="7"/>
-      <c r="N17" s="7"/>
-      <c r="O17" s="7"/>
-      <c r="P17" s="7"/>
-      <c r="Q17" s="7"/>
+      <c r="C17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6"/>
+      <c r="N17" s="6"/>
+      <c r="O17" s="6"/>
+      <c r="P17" s="6"/>
+      <c r="Q17" s="6"/>
     </row>
     <row r="18" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11">
+      <c r="A18" s="10">
         <v>9</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="7"/>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
-      <c r="L18" s="7"/>
-      <c r="M18" s="7"/>
-      <c r="N18" s="7"/>
-      <c r="O18" s="7"/>
-      <c r="P18" s="7"/>
-      <c r="Q18" s="7"/>
+      <c r="C18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="6"/>
+      <c r="L18" s="6"/>
+      <c r="M18" s="6"/>
+      <c r="N18" s="6"/>
+      <c r="O18" s="6"/>
+      <c r="P18" s="6"/>
+      <c r="Q18" s="6"/>
     </row>
     <row r="19" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="11">
+      <c r="A19" s="10">
         <v>10</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="7"/>
-      <c r="J19" s="7"/>
-      <c r="K19" s="7"/>
-      <c r="L19" s="7"/>
-      <c r="M19" s="7"/>
-      <c r="N19" s="7"/>
-      <c r="O19" s="7"/>
-      <c r="P19" s="7"/>
-      <c r="Q19" s="7"/>
+      <c r="C19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6"/>
+      <c r="N19" s="6"/>
+      <c r="O19" s="6"/>
+      <c r="P19" s="6"/>
+      <c r="Q19" s="6"/>
     </row>
     <row r="20" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="11">
+      <c r="A20" s="10">
         <v>11</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="7"/>
-      <c r="J20" s="7"/>
-      <c r="K20" s="7"/>
-      <c r="L20" s="7"/>
-      <c r="M20" s="7"/>
-      <c r="N20" s="7"/>
-      <c r="O20" s="7"/>
-      <c r="P20" s="7"/>
-      <c r="Q20" s="7"/>
+      <c r="C20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="6"/>
+      <c r="M20" s="6"/>
+      <c r="N20" s="6"/>
+      <c r="O20" s="6"/>
+      <c r="P20" s="6"/>
+      <c r="Q20" s="6"/>
     </row>
     <row r="21" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="11">
-        <v>12</v>
-      </c>
-      <c r="B21" s="4" t="s">
+      <c r="A21" s="10">
+        <v>12</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
-      <c r="M21" s="7"/>
-      <c r="N21" s="7"/>
-      <c r="O21" s="7"/>
-      <c r="P21" s="7"/>
-      <c r="Q21" s="7"/>
+      <c r="C21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6"/>
+      <c r="M21" s="6"/>
+      <c r="N21" s="6"/>
+      <c r="O21" s="6"/>
+      <c r="P21" s="6"/>
+      <c r="Q21" s="6"/>
     </row>
     <row r="22" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="11">
+      <c r="A22" s="10">
         <v>13</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="7"/>
-      <c r="L22" s="7"/>
-      <c r="M22" s="7"/>
-      <c r="N22" s="7"/>
-      <c r="O22" s="7"/>
-      <c r="P22" s="7"/>
-      <c r="Q22" s="7"/>
+      <c r="C22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6"/>
+      <c r="K22" s="6"/>
+      <c r="L22" s="6"/>
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="6"/>
+      <c r="P22" s="6"/>
+      <c r="Q22" s="6"/>
     </row>
     <row r="23" spans="1:17" ht="67.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="11">
+      <c r="A23" s="10">
         <v>14</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C23" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7"/>
-      <c r="M23" s="7"/>
-      <c r="N23" s="7"/>
-      <c r="O23" s="7"/>
-      <c r="P23" s="7"/>
-      <c r="Q23" s="7"/>
+      <c r="C23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
     </row>
     <row r="24" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="11">
+      <c r="A24" s="10">
         <v>15</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="7"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
-      <c r="L24" s="7"/>
-      <c r="M24" s="7"/>
-      <c r="N24" s="7"/>
-      <c r="O24" s="7"/>
-      <c r="P24" s="7"/>
-      <c r="Q24" s="7"/>
+      <c r="C24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="6"/>
+      <c r="K24" s="6"/>
+      <c r="L24" s="6"/>
+      <c r="M24" s="6"/>
+      <c r="N24" s="6"/>
+      <c r="O24" s="6"/>
+      <c r="P24" s="6"/>
+      <c r="Q24" s="6"/>
     </row>
     <row r="25" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="11">
+      <c r="A25" s="10">
         <v>16</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="7"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
-      <c r="L25" s="7"/>
-      <c r="M25" s="7"/>
-      <c r="N25" s="7"/>
-      <c r="O25" s="7"/>
-      <c r="P25" s="7"/>
-      <c r="Q25" s="7"/>
+      <c r="C25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
+      <c r="L25" s="6"/>
+      <c r="M25" s="6"/>
+      <c r="N25" s="6"/>
+      <c r="O25" s="6"/>
+      <c r="P25" s="6"/>
+      <c r="Q25" s="6"/>
     </row>
     <row r="26" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="11">
+      <c r="A26" s="10">
         <v>17</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
-      <c r="M26" s="7"/>
-      <c r="N26" s="7"/>
-      <c r="O26" s="7"/>
-      <c r="P26" s="7"/>
-      <c r="Q26" s="7"/>
+      <c r="C26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
+      <c r="L26" s="6"/>
+      <c r="M26" s="6"/>
+      <c r="N26" s="6"/>
+      <c r="O26" s="6"/>
+      <c r="P26" s="6"/>
+      <c r="Q26" s="6"/>
     </row>
     <row r="27" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="11">
+      <c r="A27" s="10">
         <v>18</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
-      <c r="L27" s="7"/>
-      <c r="M27" s="7"/>
-      <c r="N27" s="7"/>
-      <c r="O27" s="7"/>
-      <c r="P27" s="7"/>
-      <c r="Q27" s="7"/>
+      <c r="C27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="6"/>
+      <c r="M27" s="6"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="6"/>
+      <c r="P27" s="6"/>
+      <c r="Q27" s="6"/>
     </row>
     <row r="28" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="11">
+      <c r="A28" s="10">
         <v>19</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F28" s="4"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="7"/>
-      <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
-      <c r="L28" s="7"/>
-      <c r="M28" s="7"/>
-      <c r="N28" s="7"/>
-      <c r="O28" s="7"/>
-      <c r="P28" s="7"/>
-      <c r="Q28" s="7"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="6"/>
+      <c r="K28" s="6"/>
+      <c r="L28" s="6"/>
+      <c r="M28" s="6"/>
+      <c r="N28" s="6"/>
+      <c r="O28" s="6"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="6"/>
     </row>
     <row r="29" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="11">
+      <c r="A29" s="10">
         <v>20</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="7"/>
-      <c r="J29" s="7"/>
-      <c r="K29" s="7"/>
-      <c r="L29" s="7"/>
-      <c r="M29" s="7"/>
-      <c r="N29" s="7"/>
-      <c r="O29" s="7"/>
-      <c r="P29" s="7"/>
-      <c r="Q29" s="7"/>
+      <c r="C29" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="6"/>
+      <c r="K29" s="6"/>
+      <c r="L29" s="6"/>
+      <c r="M29" s="6"/>
+      <c r="N29" s="6"/>
+      <c r="O29" s="6"/>
+      <c r="P29" s="6"/>
+      <c r="Q29" s="6"/>
     </row>
     <row r="30" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="11">
+      <c r="A30" s="10">
         <v>21</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F30" s="4"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="7"/>
-      <c r="J30" s="7"/>
-      <c r="K30" s="7"/>
-      <c r="L30" s="7"/>
-      <c r="M30" s="7"/>
-      <c r="N30" s="7"/>
-      <c r="O30" s="7"/>
-      <c r="P30" s="7"/>
-      <c r="Q30" s="7"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
+      <c r="I30" s="6"/>
+      <c r="J30" s="6"/>
+      <c r="K30" s="6"/>
+      <c r="L30" s="6"/>
+      <c r="M30" s="6"/>
+      <c r="N30" s="6"/>
+      <c r="O30" s="6"/>
+      <c r="P30" s="6"/>
+      <c r="Q30" s="6"/>
     </row>
     <row r="31" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="11">
+      <c r="A31" s="10">
         <v>22</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="7"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
-      <c r="L31" s="7"/>
-      <c r="M31" s="7"/>
-      <c r="N31" s="7"/>
-      <c r="O31" s="7"/>
-      <c r="P31" s="7"/>
-      <c r="Q31" s="7"/>
+      <c r="C31" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="6"/>
+      <c r="N31" s="6"/>
+      <c r="O31" s="6"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="6"/>
     </row>
     <row r="32" spans="1:17" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="11">
+      <c r="A32" s="10">
         <v>23</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="C32" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="7"/>
-      <c r="J32" s="7"/>
-      <c r="K32" s="7"/>
-      <c r="L32" s="7"/>
-      <c r="M32" s="7"/>
-      <c r="N32" s="7"/>
-      <c r="O32" s="7"/>
-      <c r="P32" s="7"/>
-      <c r="Q32" s="7"/>
+      <c r="C32" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="6"/>
+      <c r="K32" s="6"/>
+      <c r="L32" s="6"/>
+      <c r="M32" s="6"/>
+      <c r="N32" s="6"/>
+      <c r="O32" s="6"/>
+      <c r="P32" s="6"/>
+      <c r="Q32" s="6"/>
     </row>
     <row r="33" spans="1:24" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="11">
+      <c r="A33" s="10">
         <v>24</v>
       </c>
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="7"/>
-      <c r="J33" s="7"/>
-      <c r="K33" s="7"/>
-      <c r="L33" s="7"/>
-      <c r="M33" s="7"/>
-      <c r="N33" s="7"/>
-      <c r="O33" s="7"/>
-      <c r="P33" s="7"/>
-      <c r="Q33" s="7"/>
+      <c r="C33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="6"/>
+      <c r="K33" s="6"/>
+      <c r="L33" s="6"/>
+      <c r="M33" s="6"/>
+      <c r="N33" s="6"/>
+      <c r="O33" s="6"/>
+      <c r="P33" s="6"/>
+      <c r="Q33" s="6"/>
     </row>
     <row r="34" spans="1:24" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="11">
+      <c r="A34" s="10">
         <v>25</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="C34" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="7"/>
-      <c r="J34" s="7"/>
-      <c r="K34" s="7"/>
-      <c r="L34" s="7"/>
-      <c r="M34" s="7"/>
-      <c r="N34" s="7"/>
-      <c r="O34" s="7"/>
-      <c r="P34" s="7"/>
-      <c r="Q34" s="7"/>
+      <c r="C34" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="6"/>
+      <c r="J34" s="6"/>
+      <c r="K34" s="6"/>
+      <c r="L34" s="6"/>
+      <c r="M34" s="6"/>
+      <c r="N34" s="6"/>
+      <c r="O34" s="6"/>
+      <c r="P34" s="6"/>
+      <c r="Q34" s="6"/>
     </row>
     <row r="35" spans="1:24" s="1" customFormat="1" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="24"/>
-      <c r="B35" s="25"/>
-      <c r="C35" s="25"/>
-      <c r="D35" s="25"/>
-      <c r="E35" s="25"/>
-      <c r="F35" s="25"/>
-      <c r="G35" s="25"/>
-      <c r="H35" s="25"/>
-      <c r="I35" s="25"/>
-      <c r="J35" s="25"/>
-      <c r="K35" s="25"/>
-      <c r="L35" s="25"/>
-      <c r="M35" s="25"/>
-      <c r="N35" s="25"/>
-      <c r="O35" s="25"/>
-      <c r="P35" s="25"/>
-      <c r="Q35" s="26"/>
+      <c r="A35" s="59"/>
+      <c r="B35" s="60"/>
+      <c r="C35" s="60"/>
+      <c r="D35" s="60"/>
+      <c r="E35" s="60"/>
+      <c r="F35" s="60"/>
+      <c r="G35" s="60"/>
+      <c r="H35" s="60"/>
+      <c r="I35" s="60"/>
+      <c r="J35" s="60"/>
+      <c r="K35" s="60"/>
+      <c r="L35" s="60"/>
+      <c r="M35" s="60"/>
+      <c r="N35" s="60"/>
+      <c r="O35" s="60"/>
+      <c r="P35" s="60"/>
+      <c r="Q35" s="61"/>
       <c r="R35"/>
       <c r="S35"/>
       <c r="T35"/>
@@ -2579,25 +2579,25 @@
       <c r="X35"/>
     </row>
     <row r="36" spans="1:24" s="1" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="27" t="s">
+      <c r="A36" s="62" t="s">
         <v>20</v>
       </c>
-      <c r="B36" s="28"/>
-      <c r="C36" s="28"/>
-      <c r="D36" s="28"/>
-      <c r="E36" s="28"/>
-      <c r="F36" s="28"/>
-      <c r="G36" s="28"/>
-      <c r="H36" s="28"/>
-      <c r="I36" s="28"/>
-      <c r="J36" s="28"/>
-      <c r="K36" s="28"/>
-      <c r="L36" s="28"/>
-      <c r="M36" s="28"/>
-      <c r="N36" s="28"/>
-      <c r="O36" s="28"/>
-      <c r="P36" s="28"/>
-      <c r="Q36" s="29"/>
+      <c r="B36" s="63"/>
+      <c r="C36" s="63"/>
+      <c r="D36" s="63"/>
+      <c r="E36" s="63"/>
+      <c r="F36" s="63"/>
+      <c r="G36" s="63"/>
+      <c r="H36" s="63"/>
+      <c r="I36" s="63"/>
+      <c r="J36" s="63"/>
+      <c r="K36" s="63"/>
+      <c r="L36" s="63"/>
+      <c r="M36" s="63"/>
+      <c r="N36" s="63"/>
+      <c r="O36" s="63"/>
+      <c r="P36" s="63"/>
+      <c r="Q36" s="64"/>
       <c r="R36"/>
       <c r="S36"/>
       <c r="T36"/>
@@ -2607,49 +2607,49 @@
       <c r="X36"/>
     </row>
     <row r="37" spans="1:24" s="1" customFormat="1" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="65" t="s">
+      <c r="A37" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B37" s="43" t="s">
+      <c r="B37" s="79" t="s">
         <v>14</v>
       </c>
-      <c r="C37" s="48" t="s">
+      <c r="C37" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="D37" s="50" t="s">
+      <c r="D37" s="81" t="s">
         <v>15</v>
       </c>
-      <c r="E37" s="45" t="s">
+      <c r="E37" s="82" t="s">
         <v>16</v>
       </c>
-      <c r="F37" s="47" t="s">
+      <c r="F37" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="G37" s="47" t="s">
+      <c r="G37" s="83" t="s">
         <v>17</v>
       </c>
-      <c r="H37" s="47"/>
-      <c r="I37" s="47" t="s">
+      <c r="H37" s="83"/>
+      <c r="I37" s="83" t="s">
         <v>26</v>
       </c>
-      <c r="J37" s="47"/>
-      <c r="K37" s="47" t="s">
+      <c r="J37" s="83"/>
+      <c r="K37" s="83" t="s">
         <v>29</v>
       </c>
-      <c r="L37" s="47"/>
-      <c r="M37" s="45" t="s">
+      <c r="L37" s="83"/>
+      <c r="M37" s="82" t="s">
         <v>28</v>
       </c>
-      <c r="N37" s="47" t="s">
+      <c r="N37" s="83" t="s">
         <v>21</v>
       </c>
-      <c r="O37" s="45" t="s">
+      <c r="O37" s="82" t="s">
         <v>23</v>
       </c>
-      <c r="P37" s="45" t="s">
+      <c r="P37" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="Q37" s="45" t="s">
+      <c r="Q37" s="82" t="s">
         <v>9</v>
       </c>
       <c r="R37"/>
@@ -2661,35 +2661,35 @@
       <c r="X37"/>
     </row>
     <row r="38" spans="1:24" s="1" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="50"/>
-      <c r="B38" s="44"/>
-      <c r="C38" s="49"/>
-      <c r="D38" s="51"/>
-      <c r="E38" s="46"/>
-      <c r="F38" s="45"/>
-      <c r="G38" s="3" t="s">
+      <c r="A38" s="81"/>
+      <c r="B38" s="84"/>
+      <c r="C38" s="85"/>
+      <c r="D38" s="86"/>
+      <c r="E38" s="87"/>
+      <c r="F38" s="82"/>
+      <c r="G38" s="88" t="s">
         <v>18</v>
       </c>
-      <c r="H38" s="3" t="s">
+      <c r="H38" s="88" t="s">
         <v>19</v>
       </c>
-      <c r="I38" s="3" t="s">
+      <c r="I38" s="88" t="s">
         <v>18</v>
       </c>
-      <c r="J38" s="3" t="s">
+      <c r="J38" s="88" t="s">
         <v>19</v>
       </c>
-      <c r="K38" s="3" t="s">
+      <c r="K38" s="88" t="s">
         <v>18</v>
       </c>
-      <c r="L38" s="3" t="s">
+      <c r="L38" s="88" t="s">
         <v>19</v>
       </c>
-      <c r="M38" s="46"/>
-      <c r="N38" s="45"/>
-      <c r="O38" s="46"/>
-      <c r="P38" s="46"/>
-      <c r="Q38" s="46"/>
+      <c r="M38" s="87"/>
+      <c r="N38" s="82"/>
+      <c r="O38" s="87"/>
+      <c r="P38" s="87"/>
+      <c r="Q38" s="87"/>
       <c r="R38"/>
       <c r="S38"/>
       <c r="T38"/>
@@ -2699,23 +2699,23 @@
       <c r="X38"/>
     </row>
     <row r="39" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="17"/>
-      <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="17"/>
-      <c r="F39" s="17"/>
-      <c r="G39" s="17"/>
-      <c r="H39" s="17"/>
-      <c r="I39" s="17"/>
-      <c r="J39" s="17"/>
-      <c r="K39" s="17"/>
-      <c r="L39" s="17"/>
-      <c r="M39" s="17"/>
-      <c r="N39" s="17"/>
-      <c r="O39" s="17"/>
-      <c r="P39" s="17"/>
-      <c r="Q39" s="17"/>
+      <c r="A39" s="16"/>
+      <c r="B39" s="16"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="16"/>
+      <c r="H39" s="16"/>
+      <c r="I39" s="16"/>
+      <c r="J39" s="16"/>
+      <c r="K39" s="16"/>
+      <c r="L39" s="16"/>
+      <c r="M39" s="16"/>
+      <c r="N39" s="16"/>
+      <c r="O39" s="16"/>
+      <c r="P39" s="16"/>
+      <c r="Q39" s="16"/>
       <c r="R39"/>
       <c r="S39"/>
       <c r="T39"/>
@@ -2725,23 +2725,23 @@
       <c r="X39"/>
     </row>
     <row r="40" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="17"/>
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="17"/>
-      <c r="E40" s="17"/>
-      <c r="F40" s="17"/>
-      <c r="G40" s="17"/>
-      <c r="H40" s="17"/>
-      <c r="I40" s="17"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="17"/>
-      <c r="L40" s="17"/>
-      <c r="M40" s="17"/>
-      <c r="N40" s="17"/>
-      <c r="O40" s="17"/>
-      <c r="P40" s="17"/>
-      <c r="Q40" s="17"/>
+      <c r="A40" s="16"/>
+      <c r="B40" s="16"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
+      <c r="I40" s="16"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="16"/>
+      <c r="L40" s="16"/>
+      <c r="M40" s="16"/>
+      <c r="N40" s="16"/>
+      <c r="O40" s="16"/>
+      <c r="P40" s="16"/>
+      <c r="Q40" s="16"/>
       <c r="R40"/>
       <c r="S40"/>
       <c r="T40"/>
@@ -2751,23 +2751,23 @@
       <c r="X40"/>
     </row>
     <row r="41" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="17"/>
-      <c r="B41" s="17"/>
-      <c r="C41" s="17"/>
-      <c r="D41" s="17"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="17"/>
-      <c r="I41" s="17"/>
-      <c r="J41" s="17"/>
-      <c r="K41" s="17"/>
-      <c r="L41" s="17"/>
-      <c r="M41" s="17"/>
-      <c r="N41" s="17"/>
-      <c r="O41" s="17"/>
-      <c r="P41" s="17"/>
-      <c r="Q41" s="17"/>
+      <c r="A41" s="16"/>
+      <c r="B41" s="16"/>
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
+      <c r="E41" s="16"/>
+      <c r="F41" s="16"/>
+      <c r="G41" s="16"/>
+      <c r="H41" s="16"/>
+      <c r="I41" s="16"/>
+      <c r="J41" s="16"/>
+      <c r="K41" s="16"/>
+      <c r="L41" s="16"/>
+      <c r="M41" s="16"/>
+      <c r="N41" s="16"/>
+      <c r="O41" s="16"/>
+      <c r="P41" s="16"/>
+      <c r="Q41" s="16"/>
       <c r="R41"/>
       <c r="S41"/>
       <c r="T41"/>
@@ -2777,23 +2777,23 @@
       <c r="X41"/>
     </row>
     <row r="42" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="17"/>
-      <c r="B42" s="17"/>
-      <c r="C42" s="17"/>
-      <c r="D42" s="17"/>
-      <c r="E42" s="17"/>
-      <c r="F42" s="17"/>
-      <c r="G42" s="17"/>
-      <c r="H42" s="17"/>
-      <c r="I42" s="17"/>
-      <c r="J42" s="17"/>
-      <c r="K42" s="17"/>
-      <c r="L42" s="17"/>
-      <c r="M42" s="17"/>
-      <c r="N42" s="17"/>
-      <c r="O42" s="17"/>
-      <c r="P42" s="17"/>
-      <c r="Q42" s="17"/>
+      <c r="A42" s="16"/>
+      <c r="B42" s="16"/>
+      <c r="C42" s="16"/>
+      <c r="D42" s="16"/>
+      <c r="E42" s="16"/>
+      <c r="F42" s="16"/>
+      <c r="G42" s="16"/>
+      <c r="H42" s="16"/>
+      <c r="I42" s="16"/>
+      <c r="J42" s="16"/>
+      <c r="K42" s="16"/>
+      <c r="L42" s="16"/>
+      <c r="M42" s="16"/>
+      <c r="N42" s="16"/>
+      <c r="O42" s="16"/>
+      <c r="P42" s="16"/>
+      <c r="Q42" s="16"/>
       <c r="R42"/>
       <c r="S42"/>
       <c r="T42"/>
@@ -2803,23 +2803,23 @@
       <c r="X42"/>
     </row>
     <row r="43" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="17"/>
-      <c r="B43" s="17"/>
-      <c r="C43" s="17"/>
-      <c r="D43" s="17"/>
-      <c r="E43" s="17"/>
-      <c r="F43" s="17"/>
-      <c r="G43" s="17"/>
-      <c r="H43" s="17"/>
-      <c r="I43" s="17"/>
-      <c r="J43" s="17"/>
-      <c r="K43" s="17"/>
-      <c r="L43" s="17"/>
-      <c r="M43" s="17"/>
-      <c r="N43" s="17"/>
-      <c r="O43" s="17"/>
-      <c r="P43" s="17"/>
-      <c r="Q43" s="17"/>
+      <c r="A43" s="16"/>
+      <c r="B43" s="16"/>
+      <c r="C43" s="16"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="16"/>
+      <c r="G43" s="16"/>
+      <c r="H43" s="16"/>
+      <c r="I43" s="16"/>
+      <c r="J43" s="16"/>
+      <c r="K43" s="16"/>
+      <c r="L43" s="16"/>
+      <c r="M43" s="16"/>
+      <c r="N43" s="16"/>
+      <c r="O43" s="16"/>
+      <c r="P43" s="16"/>
+      <c r="Q43" s="16"/>
       <c r="R43"/>
       <c r="S43"/>
       <c r="T43"/>
@@ -2829,23 +2829,23 @@
       <c r="X43"/>
     </row>
     <row r="44" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="17"/>
-      <c r="B44" s="17"/>
-      <c r="C44" s="17"/>
-      <c r="D44" s="17"/>
-      <c r="E44" s="17"/>
-      <c r="F44" s="17"/>
-      <c r="G44" s="17"/>
-      <c r="H44" s="17"/>
-      <c r="I44" s="17"/>
-      <c r="J44" s="17"/>
-      <c r="K44" s="17"/>
-      <c r="L44" s="17"/>
-      <c r="M44" s="17"/>
-      <c r="N44" s="17"/>
-      <c r="O44" s="17"/>
-      <c r="P44" s="17"/>
-      <c r="Q44" s="17"/>
+      <c r="A44" s="16"/>
+      <c r="B44" s="16"/>
+      <c r="C44" s="16"/>
+      <c r="D44" s="16"/>
+      <c r="E44" s="16"/>
+      <c r="F44" s="16"/>
+      <c r="G44" s="16"/>
+      <c r="H44" s="16"/>
+      <c r="I44" s="16"/>
+      <c r="J44" s="16"/>
+      <c r="K44" s="16"/>
+      <c r="L44" s="16"/>
+      <c r="M44" s="16"/>
+      <c r="N44" s="16"/>
+      <c r="O44" s="16"/>
+      <c r="P44" s="16"/>
+      <c r="Q44" s="16"/>
       <c r="R44"/>
       <c r="S44"/>
       <c r="T44"/>
@@ -2855,23 +2855,23 @@
       <c r="X44"/>
     </row>
     <row r="45" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="17"/>
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
-      <c r="L45" s="17"/>
-      <c r="M45" s="17"/>
-      <c r="N45" s="17"/>
-      <c r="O45" s="17"/>
-      <c r="P45" s="17"/>
-      <c r="Q45" s="17"/>
+      <c r="A45" s="16"/>
+      <c r="B45" s="16"/>
+      <c r="C45" s="16"/>
+      <c r="D45" s="16"/>
+      <c r="E45" s="16"/>
+      <c r="F45" s="16"/>
+      <c r="G45" s="16"/>
+      <c r="H45" s="16"/>
+      <c r="I45" s="16"/>
+      <c r="J45" s="16"/>
+      <c r="K45" s="16"/>
+      <c r="L45" s="16"/>
+      <c r="M45" s="16"/>
+      <c r="N45" s="16"/>
+      <c r="O45" s="16"/>
+      <c r="P45" s="16"/>
+      <c r="Q45" s="16"/>
       <c r="R45"/>
       <c r="S45"/>
       <c r="T45"/>
@@ -2881,23 +2881,23 @@
       <c r="X45"/>
     </row>
     <row r="46" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="17"/>
-      <c r="B46" s="17"/>
-      <c r="C46" s="17"/>
-      <c r="D46" s="17"/>
-      <c r="E46" s="17"/>
-      <c r="F46" s="17"/>
-      <c r="G46" s="17"/>
-      <c r="H46" s="17"/>
-      <c r="I46" s="17"/>
-      <c r="J46" s="17"/>
-      <c r="K46" s="17"/>
-      <c r="L46" s="17"/>
-      <c r="M46" s="17"/>
-      <c r="N46" s="17"/>
-      <c r="O46" s="17"/>
-      <c r="P46" s="17"/>
-      <c r="Q46" s="17"/>
+      <c r="A46" s="16"/>
+      <c r="B46" s="16"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="16"/>
+      <c r="F46" s="16"/>
+      <c r="G46" s="16"/>
+      <c r="H46" s="16"/>
+      <c r="I46" s="16"/>
+      <c r="J46" s="16"/>
+      <c r="K46" s="16"/>
+      <c r="L46" s="16"/>
+      <c r="M46" s="16"/>
+      <c r="N46" s="16"/>
+      <c r="O46" s="16"/>
+      <c r="P46" s="16"/>
+      <c r="Q46" s="16"/>
       <c r="R46"/>
       <c r="S46"/>
       <c r="T46"/>
@@ -2907,23 +2907,23 @@
       <c r="X46"/>
     </row>
     <row r="47" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="17"/>
-      <c r="B47" s="17"/>
-      <c r="C47" s="17"/>
-      <c r="D47" s="17"/>
-      <c r="E47" s="17"/>
-      <c r="F47" s="17"/>
-      <c r="G47" s="17"/>
-      <c r="H47" s="17"/>
-      <c r="I47" s="17"/>
-      <c r="J47" s="17"/>
-      <c r="K47" s="17"/>
-      <c r="L47" s="17"/>
-      <c r="M47" s="17"/>
-      <c r="N47" s="17"/>
-      <c r="O47" s="17"/>
-      <c r="P47" s="17"/>
-      <c r="Q47" s="17"/>
+      <c r="A47" s="16"/>
+      <c r="B47" s="16"/>
+      <c r="C47" s="16"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="16"/>
+      <c r="G47" s="16"/>
+      <c r="H47" s="16"/>
+      <c r="I47" s="16"/>
+      <c r="J47" s="16"/>
+      <c r="K47" s="16"/>
+      <c r="L47" s="16"/>
+      <c r="M47" s="16"/>
+      <c r="N47" s="16"/>
+      <c r="O47" s="16"/>
+      <c r="P47" s="16"/>
+      <c r="Q47" s="16"/>
       <c r="R47"/>
       <c r="S47"/>
       <c r="T47"/>
@@ -2933,23 +2933,23 @@
       <c r="X47"/>
     </row>
     <row r="48" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="17"/>
-      <c r="B48" s="17"/>
-      <c r="C48" s="17"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="17"/>
-      <c r="F48" s="17"/>
-      <c r="G48" s="17"/>
-      <c r="H48" s="17"/>
-      <c r="I48" s="17"/>
-      <c r="J48" s="17"/>
-      <c r="K48" s="17"/>
-      <c r="L48" s="17"/>
-      <c r="M48" s="17"/>
-      <c r="N48" s="17"/>
-      <c r="O48" s="17"/>
-      <c r="P48" s="17"/>
-      <c r="Q48" s="17"/>
+      <c r="A48" s="16"/>
+      <c r="B48" s="16"/>
+      <c r="C48" s="16"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
+      <c r="F48" s="16"/>
+      <c r="G48" s="16"/>
+      <c r="H48" s="16"/>
+      <c r="I48" s="16"/>
+      <c r="J48" s="16"/>
+      <c r="K48" s="16"/>
+      <c r="L48" s="16"/>
+      <c r="M48" s="16"/>
+      <c r="N48" s="16"/>
+      <c r="O48" s="16"/>
+      <c r="P48" s="16"/>
+      <c r="Q48" s="16"/>
       <c r="R48"/>
       <c r="S48"/>
       <c r="T48"/>
@@ -2959,23 +2959,23 @@
       <c r="X48"/>
     </row>
     <row r="49" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="17"/>
-      <c r="B49" s="17"/>
-      <c r="C49" s="17"/>
-      <c r="D49" s="17"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="17"/>
-      <c r="H49" s="17"/>
-      <c r="I49" s="17"/>
-      <c r="J49" s="17"/>
-      <c r="K49" s="17"/>
-      <c r="L49" s="17"/>
-      <c r="M49" s="17"/>
-      <c r="N49" s="17"/>
-      <c r="O49" s="17"/>
-      <c r="P49" s="17"/>
-      <c r="Q49" s="17"/>
+      <c r="A49" s="16"/>
+      <c r="B49" s="16"/>
+      <c r="C49" s="16"/>
+      <c r="D49" s="16"/>
+      <c r="E49" s="16"/>
+      <c r="F49" s="16"/>
+      <c r="G49" s="16"/>
+      <c r="H49" s="16"/>
+      <c r="I49" s="16"/>
+      <c r="J49" s="16"/>
+      <c r="K49" s="16"/>
+      <c r="L49" s="16"/>
+      <c r="M49" s="16"/>
+      <c r="N49" s="16"/>
+      <c r="O49" s="16"/>
+      <c r="P49" s="16"/>
+      <c r="Q49" s="16"/>
       <c r="R49"/>
       <c r="S49"/>
       <c r="T49"/>
@@ -2985,23 +2985,23 @@
       <c r="X49"/>
     </row>
     <row r="50" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="17"/>
-      <c r="B50" s="17"/>
-      <c r="C50" s="17"/>
-      <c r="D50" s="17"/>
-      <c r="E50" s="17"/>
-      <c r="F50" s="17"/>
-      <c r="G50" s="17"/>
-      <c r="H50" s="17"/>
-      <c r="I50" s="17"/>
-      <c r="J50" s="17"/>
-      <c r="K50" s="17"/>
-      <c r="L50" s="17"/>
-      <c r="M50" s="17"/>
-      <c r="N50" s="17"/>
-      <c r="O50" s="17"/>
-      <c r="P50" s="17"/>
-      <c r="Q50" s="17"/>
+      <c r="A50" s="16"/>
+      <c r="B50" s="16"/>
+      <c r="C50" s="16"/>
+      <c r="D50" s="16"/>
+      <c r="E50" s="16"/>
+      <c r="F50" s="16"/>
+      <c r="G50" s="16"/>
+      <c r="H50" s="16"/>
+      <c r="I50" s="16"/>
+      <c r="J50" s="16"/>
+      <c r="K50" s="16"/>
+      <c r="L50" s="16"/>
+      <c r="M50" s="16"/>
+      <c r="N50" s="16"/>
+      <c r="O50" s="16"/>
+      <c r="P50" s="16"/>
+      <c r="Q50" s="16"/>
       <c r="R50"/>
       <c r="S50"/>
       <c r="T50"/>
@@ -3011,23 +3011,23 @@
       <c r="X50"/>
     </row>
     <row r="51" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="17"/>
-      <c r="B51" s="17"/>
-      <c r="C51" s="17"/>
-      <c r="D51" s="17"/>
-      <c r="E51" s="17"/>
-      <c r="F51" s="17"/>
-      <c r="G51" s="17"/>
-      <c r="H51" s="17"/>
-      <c r="I51" s="17"/>
-      <c r="J51" s="17"/>
-      <c r="K51" s="17"/>
-      <c r="L51" s="17"/>
-      <c r="M51" s="17"/>
-      <c r="N51" s="17"/>
-      <c r="O51" s="17"/>
-      <c r="P51" s="17"/>
-      <c r="Q51" s="17"/>
+      <c r="A51" s="16"/>
+      <c r="B51" s="16"/>
+      <c r="C51" s="16"/>
+      <c r="D51" s="16"/>
+      <c r="E51" s="16"/>
+      <c r="F51" s="16"/>
+      <c r="G51" s="16"/>
+      <c r="H51" s="16"/>
+      <c r="I51" s="16"/>
+      <c r="J51" s="16"/>
+      <c r="K51" s="16"/>
+      <c r="L51" s="16"/>
+      <c r="M51" s="16"/>
+      <c r="N51" s="16"/>
+      <c r="O51" s="16"/>
+      <c r="P51" s="16"/>
+      <c r="Q51" s="16"/>
       <c r="R51"/>
       <c r="S51"/>
       <c r="T51"/>
@@ -3037,23 +3037,23 @@
       <c r="X51"/>
     </row>
     <row r="52" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="17"/>
-      <c r="B52" s="17"/>
-      <c r="C52" s="17"/>
-      <c r="D52" s="17"/>
-      <c r="E52" s="17"/>
-      <c r="F52" s="17"/>
-      <c r="G52" s="17"/>
-      <c r="H52" s="17"/>
-      <c r="I52" s="17"/>
-      <c r="J52" s="17"/>
-      <c r="K52" s="17"/>
-      <c r="L52" s="17"/>
-      <c r="M52" s="17"/>
-      <c r="N52" s="17"/>
-      <c r="O52" s="17"/>
-      <c r="P52" s="17"/>
-      <c r="Q52" s="17"/>
+      <c r="A52" s="16"/>
+      <c r="B52" s="16"/>
+      <c r="C52" s="16"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
+      <c r="F52" s="16"/>
+      <c r="G52" s="16"/>
+      <c r="H52" s="16"/>
+      <c r="I52" s="16"/>
+      <c r="J52" s="16"/>
+      <c r="K52" s="16"/>
+      <c r="L52" s="16"/>
+      <c r="M52" s="16"/>
+      <c r="N52" s="16"/>
+      <c r="O52" s="16"/>
+      <c r="P52" s="16"/>
+      <c r="Q52" s="16"/>
       <c r="R52"/>
       <c r="S52"/>
       <c r="T52"/>
@@ -3063,23 +3063,23 @@
       <c r="X52"/>
     </row>
     <row r="53" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="17"/>
-      <c r="B53" s="17"/>
-      <c r="C53" s="17"/>
-      <c r="D53" s="17"/>
-      <c r="E53" s="17"/>
-      <c r="F53" s="17"/>
-      <c r="G53" s="17"/>
-      <c r="H53" s="17"/>
-      <c r="I53" s="17"/>
-      <c r="J53" s="17"/>
-      <c r="K53" s="17"/>
-      <c r="L53" s="17"/>
-      <c r="M53" s="17"/>
-      <c r="N53" s="17"/>
-      <c r="O53" s="17"/>
-      <c r="P53" s="17"/>
-      <c r="Q53" s="17"/>
+      <c r="A53" s="16"/>
+      <c r="B53" s="16"/>
+      <c r="C53" s="16"/>
+      <c r="D53" s="16"/>
+      <c r="E53" s="16"/>
+      <c r="F53" s="16"/>
+      <c r="G53" s="16"/>
+      <c r="H53" s="16"/>
+      <c r="I53" s="16"/>
+      <c r="J53" s="16"/>
+      <c r="K53" s="16"/>
+      <c r="L53" s="16"/>
+      <c r="M53" s="16"/>
+      <c r="N53" s="16"/>
+      <c r="O53" s="16"/>
+      <c r="P53" s="16"/>
+      <c r="Q53" s="16"/>
       <c r="R53"/>
       <c r="S53"/>
       <c r="T53"/>
@@ -3089,23 +3089,23 @@
       <c r="X53"/>
     </row>
     <row r="54" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="18"/>
-      <c r="B54" s="19"/>
-      <c r="C54" s="19"/>
-      <c r="D54" s="19"/>
-      <c r="E54" s="19"/>
-      <c r="F54" s="19"/>
-      <c r="G54" s="20"/>
-      <c r="H54" s="21"/>
-      <c r="I54" s="20"/>
-      <c r="J54" s="21"/>
-      <c r="K54" s="22"/>
-      <c r="L54" s="22"/>
-      <c r="M54" s="17"/>
-      <c r="N54" s="17"/>
-      <c r="O54" s="17"/>
-      <c r="P54" s="17"/>
-      <c r="Q54" s="23"/>
+      <c r="A54" s="17"/>
+      <c r="B54" s="18"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="18"/>
+      <c r="F54" s="18"/>
+      <c r="G54" s="19"/>
+      <c r="H54" s="20"/>
+      <c r="I54" s="19"/>
+      <c r="J54" s="20"/>
+      <c r="K54" s="21"/>
+      <c r="L54" s="21"/>
+      <c r="M54" s="16"/>
+      <c r="N54" s="16"/>
+      <c r="O54" s="16"/>
+      <c r="P54" s="16"/>
+      <c r="Q54" s="22"/>
       <c r="R54"/>
       <c r="S54"/>
       <c r="T54"/>
@@ -3115,23 +3115,23 @@
       <c r="X54"/>
     </row>
     <row r="55" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="18"/>
-      <c r="B55" s="19"/>
-      <c r="C55" s="19"/>
-      <c r="D55" s="19"/>
-      <c r="E55" s="19"/>
-      <c r="F55" s="19"/>
-      <c r="G55" s="20"/>
-      <c r="H55" s="21"/>
-      <c r="I55" s="20"/>
-      <c r="J55" s="21"/>
-      <c r="K55" s="22"/>
-      <c r="L55" s="22"/>
-      <c r="M55" s="17"/>
-      <c r="N55" s="17"/>
-      <c r="O55" s="17"/>
-      <c r="P55" s="17"/>
-      <c r="Q55" s="23"/>
+      <c r="A55" s="17"/>
+      <c r="B55" s="18"/>
+      <c r="C55" s="18"/>
+      <c r="D55" s="18"/>
+      <c r="E55" s="18"/>
+      <c r="F55" s="18"/>
+      <c r="G55" s="19"/>
+      <c r="H55" s="20"/>
+      <c r="I55" s="19"/>
+      <c r="J55" s="20"/>
+      <c r="K55" s="21"/>
+      <c r="L55" s="21"/>
+      <c r="M55" s="16"/>
+      <c r="N55" s="16"/>
+      <c r="O55" s="16"/>
+      <c r="P55" s="16"/>
+      <c r="Q55" s="22"/>
       <c r="R55"/>
       <c r="S55"/>
       <c r="T55"/>
@@ -3141,23 +3141,23 @@
       <c r="X55"/>
     </row>
     <row r="56" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="18"/>
-      <c r="B56" s="19"/>
-      <c r="C56" s="19"/>
-      <c r="D56" s="19"/>
-      <c r="E56" s="19"/>
-      <c r="F56" s="19"/>
-      <c r="G56" s="20"/>
-      <c r="H56" s="21"/>
-      <c r="I56" s="20"/>
-      <c r="J56" s="21"/>
-      <c r="K56" s="22"/>
-      <c r="L56" s="22"/>
-      <c r="M56" s="17"/>
-      <c r="N56" s="17"/>
-      <c r="O56" s="17"/>
-      <c r="P56" s="17"/>
-      <c r="Q56" s="23"/>
+      <c r="A56" s="17"/>
+      <c r="B56" s="18"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="18"/>
+      <c r="F56" s="18"/>
+      <c r="G56" s="19"/>
+      <c r="H56" s="20"/>
+      <c r="I56" s="19"/>
+      <c r="J56" s="20"/>
+      <c r="K56" s="21"/>
+      <c r="L56" s="21"/>
+      <c r="M56" s="16"/>
+      <c r="N56" s="16"/>
+      <c r="O56" s="16"/>
+      <c r="P56" s="16"/>
+      <c r="Q56" s="22"/>
       <c r="R56"/>
       <c r="S56"/>
       <c r="T56"/>
@@ -3167,23 +3167,23 @@
       <c r="X56"/>
     </row>
     <row r="57" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="18"/>
-      <c r="B57" s="19"/>
-      <c r="C57" s="19"/>
-      <c r="D57" s="19"/>
-      <c r="E57" s="19"/>
-      <c r="F57" s="19"/>
-      <c r="G57" s="20"/>
-      <c r="H57" s="21"/>
-      <c r="I57" s="20"/>
-      <c r="J57" s="21"/>
-      <c r="K57" s="22"/>
-      <c r="L57" s="22"/>
-      <c r="M57" s="17"/>
-      <c r="N57" s="17"/>
-      <c r="O57" s="17"/>
-      <c r="P57" s="17"/>
-      <c r="Q57" s="23"/>
+      <c r="A57" s="17"/>
+      <c r="B57" s="18"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="18"/>
+      <c r="F57" s="18"/>
+      <c r="G57" s="19"/>
+      <c r="H57" s="20"/>
+      <c r="I57" s="19"/>
+      <c r="J57" s="20"/>
+      <c r="K57" s="21"/>
+      <c r="L57" s="21"/>
+      <c r="M57" s="16"/>
+      <c r="N57" s="16"/>
+      <c r="O57" s="16"/>
+      <c r="P57" s="16"/>
+      <c r="Q57" s="22"/>
       <c r="R57"/>
       <c r="S57"/>
       <c r="T57"/>
@@ -3193,23 +3193,23 @@
       <c r="X57"/>
     </row>
     <row r="58" spans="1:24" s="1" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="18"/>
-      <c r="B58" s="19"/>
-      <c r="C58" s="19"/>
-      <c r="D58" s="19"/>
-      <c r="E58" s="19"/>
-      <c r="F58" s="19"/>
-      <c r="G58" s="20"/>
-      <c r="H58" s="21"/>
-      <c r="I58" s="20"/>
-      <c r="J58" s="21"/>
-      <c r="K58" s="22"/>
-      <c r="L58" s="22"/>
-      <c r="M58" s="17"/>
-      <c r="N58" s="17"/>
-      <c r="O58" s="17"/>
-      <c r="P58" s="17"/>
-      <c r="Q58" s="23"/>
+      <c r="A58" s="17"/>
+      <c r="B58" s="18"/>
+      <c r="C58" s="18"/>
+      <c r="D58" s="18"/>
+      <c r="E58" s="18"/>
+      <c r="F58" s="18"/>
+      <c r="G58" s="19"/>
+      <c r="H58" s="20"/>
+      <c r="I58" s="19"/>
+      <c r="J58" s="20"/>
+      <c r="K58" s="21"/>
+      <c r="L58" s="21"/>
+      <c r="M58" s="16"/>
+      <c r="N58" s="16"/>
+      <c r="O58" s="16"/>
+      <c r="P58" s="16"/>
+      <c r="Q58" s="22"/>
       <c r="R58"/>
       <c r="S58"/>
       <c r="T58"/>
@@ -3219,114 +3219,122 @@
       <c r="X58"/>
     </row>
     <row r="59" spans="1:24" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="54"/>
-      <c r="B59" s="55"/>
-      <c r="C59" s="55"/>
-      <c r="D59" s="55"/>
-      <c r="E59" s="55"/>
-      <c r="F59" s="55"/>
-      <c r="G59" s="55"/>
-      <c r="H59" s="55"/>
-      <c r="I59" s="55"/>
-      <c r="J59" s="55"/>
-      <c r="K59" s="55"/>
-      <c r="L59" s="55"/>
-      <c r="M59" s="55"/>
-      <c r="N59" s="55"/>
-      <c r="O59" s="55"/>
-      <c r="P59" s="55"/>
-      <c r="Q59" s="56"/>
+      <c r="A59" s="43"/>
+      <c r="B59" s="44"/>
+      <c r="C59" s="44"/>
+      <c r="D59" s="44"/>
+      <c r="E59" s="44"/>
+      <c r="F59" s="44"/>
+      <c r="G59" s="44"/>
+      <c r="H59" s="44"/>
+      <c r="I59" s="44"/>
+      <c r="J59" s="44"/>
+      <c r="K59" s="44"/>
+      <c r="L59" s="44"/>
+      <c r="M59" s="44"/>
+      <c r="N59" s="44"/>
+      <c r="O59" s="44"/>
+      <c r="P59" s="44"/>
+      <c r="Q59" s="45"/>
       <c r="R59" s="2"/>
     </row>
     <row r="60" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="57" t="s">
+      <c r="A60" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="B60" s="58"/>
-      <c r="C60" s="58"/>
-      <c r="D60" s="58"/>
-      <c r="E60" s="58"/>
-      <c r="F60" s="58"/>
-      <c r="G60" s="59"/>
-      <c r="H60" s="59"/>
-      <c r="I60" s="59"/>
-      <c r="J60" s="59"/>
-      <c r="K60" s="59"/>
-      <c r="L60" s="59"/>
-      <c r="M60" s="59"/>
-      <c r="N60" s="59"/>
-      <c r="O60" s="59"/>
-      <c r="P60" s="59"/>
-      <c r="Q60" s="60"/>
+      <c r="B60" s="47"/>
+      <c r="C60" s="47"/>
+      <c r="D60" s="47"/>
+      <c r="E60" s="47"/>
+      <c r="F60" s="47"/>
+      <c r="G60" s="48"/>
+      <c r="H60" s="48"/>
+      <c r="I60" s="48"/>
+      <c r="J60" s="48"/>
+      <c r="K60" s="48"/>
+      <c r="L60" s="48"/>
+      <c r="M60" s="48"/>
+      <c r="N60" s="48"/>
+      <c r="O60" s="48"/>
+      <c r="P60" s="48"/>
+      <c r="Q60" s="49"/>
       <c r="R60" s="2"/>
     </row>
     <row r="61" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="61" t="s">
+      <c r="A61" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="B61" s="62"/>
-      <c r="C61" s="62"/>
-      <c r="D61" s="62" t="s">
+      <c r="B61" s="51"/>
+      <c r="C61" s="51"/>
+      <c r="D61" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="E61" s="62"/>
-      <c r="F61" s="62"/>
-      <c r="G61" s="14" t="s">
+      <c r="E61" s="51"/>
+      <c r="F61" s="51"/>
+      <c r="G61" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="H61" s="14" t="s">
+      <c r="H61" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="I61" s="14" t="s">
+      <c r="I61" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="J61" s="14" t="s">
+      <c r="J61" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="K61" s="16"/>
-      <c r="L61" s="14"/>
-      <c r="M61" s="63"/>
-      <c r="N61" s="64"/>
-      <c r="O61" s="64"/>
+      <c r="K61" s="15"/>
+      <c r="L61" s="13"/>
+      <c r="M61" s="52"/>
+      <c r="N61" s="53"/>
+      <c r="O61" s="53"/>
       <c r="R61" s="2"/>
     </row>
     <row r="62" spans="1:24" ht="156.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="38" t="s">
+      <c r="A62" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="B62" s="39"/>
-      <c r="C62" s="40"/>
-      <c r="D62" s="41"/>
-      <c r="E62" s="41"/>
-      <c r="F62" s="41"/>
-      <c r="G62" s="6" t="s">
+      <c r="B62" s="55"/>
+      <c r="C62" s="56"/>
+      <c r="D62" s="57"/>
+      <c r="E62" s="57"/>
+      <c r="F62" s="57"/>
+      <c r="G62" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="H62" s="15"/>
-      <c r="I62" s="6" t="s">
+      <c r="H62" s="14"/>
+      <c r="I62" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="J62" s="15"/>
-      <c r="K62" s="15"/>
-      <c r="L62" s="15"/>
-      <c r="M62" s="42"/>
-      <c r="N62" s="39"/>
-      <c r="O62" s="39"/>
-      <c r="P62" s="52"/>
-      <c r="Q62" s="53"/>
+      <c r="J62" s="14"/>
+      <c r="K62" s="14"/>
+      <c r="L62" s="14"/>
+      <c r="M62" s="58"/>
+      <c r="N62" s="55"/>
+      <c r="O62" s="55"/>
+      <c r="P62" s="41"/>
+      <c r="Q62" s="42"/>
       <c r="R62" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="A4:Q4"/>
-    <mergeCell ref="H5:N6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="O5:O6"/>
-    <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:N2"/>
-    <mergeCell ref="O2:Q2"/>
-    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="A35:Q35"/>
+    <mergeCell ref="A36:Q36"/>
+    <mergeCell ref="A7:Q7"/>
+    <mergeCell ref="A8:Q8"/>
+    <mergeCell ref="A5:B6"/>
+    <mergeCell ref="P5:P6"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="E5:G6"/>
+    <mergeCell ref="A62:C62"/>
+    <mergeCell ref="D62:F62"/>
+    <mergeCell ref="M62:O62"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="D37:D38"/>
     <mergeCell ref="P62:Q62"/>
     <mergeCell ref="P37:P38"/>
     <mergeCell ref="Q37:Q38"/>
@@ -3343,23 +3351,15 @@
     <mergeCell ref="N37:N38"/>
     <mergeCell ref="O37:O38"/>
     <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A62:C62"/>
-    <mergeCell ref="D62:F62"/>
-    <mergeCell ref="M62:O62"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="A35:Q35"/>
-    <mergeCell ref="A36:Q36"/>
-    <mergeCell ref="A7:Q7"/>
-    <mergeCell ref="A8:Q8"/>
-    <mergeCell ref="A5:B6"/>
-    <mergeCell ref="P5:P6"/>
-    <mergeCell ref="Q5:Q6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="E5:G6"/>
+    <mergeCell ref="A4:Q4"/>
+    <mergeCell ref="H5:N6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:N2"/>
+    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="A3:Q3"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="22" fitToHeight="0" orientation="landscape" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>